<commit_message>
File-watcher çift log yazma sorunu düzeltildi
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF93247-4FA4-4597-8E81-A6B6BDC0AF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208A5350-B914-4274-815F-CD61C8062ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,15 +74,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>102781</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>170548</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>123449</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -105,8 +105,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="15952381" cy="7219048"/>
+          <a:off x="1" y="0"/>
+          <a:ext cx="14144248" cy="6400800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Temizlik: Gereksiz test ve debug dosyaları silindi
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208A5350-B914-4274-815F-CD61C8062ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F3A67A-D4F5-4C27-8C95-D08DB3A23160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,22 +74,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>123449</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>588571</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>84857</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Resim 1">
+        <xdr:cNvPr id="3" name="Resim 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12DEFF5D-66C8-D6ED-C117-0DB6D34036AB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D8796FC-B10F-5955-C878-095498D12609}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -105,8 +105,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1" y="0"/>
-          <a:ext cx="14144248" cy="6400800"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="15828571" cy="6942857"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Add colored headers and consistent zoom controls to all Excel pages
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F3A67A-D4F5-4C27-8C95-D08DB3A23160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320DAB21-05C6-4465-B214-125F2A5D090C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,16 +80,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>588571</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>84857</xdr:rowOff>
+      <xdr:colOff>569524</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>180024</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Resim 2">
+        <xdr:cNvPr id="2" name="Resim 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D8796FC-B10F-5955-C878-095498D12609}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEDA1A42-1558-E355-55C2-A07DCA648201}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -106,7 +106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="15828571" cy="6942857"/>
+          <a:ext cx="15809524" cy="7609524"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Move notifications, messages, and announcements to header - remove from main menu - add home button
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320DAB21-05C6-4465-B214-125F2A5D090C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCBDDEA-5F3F-46FF-9374-DF40C93EF66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,17 +79,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>569524</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>180024</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>150628</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>189571</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Resim 1">
+        <xdr:cNvPr id="3" name="Resim 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEDA1A42-1558-E355-55C2-A07DCA648201}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24B9654B-92DF-32B6-2AA8-6ACC84647DE6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -106,7 +106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="15809524" cy="7609524"/>
+          <a:ext cx="14171428" cy="7428571"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Add DCS A012, A021, B012, B021 report pages with submenu navigation
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCBDDEA-5F3F-46FF-9374-DF40C93EF66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626D5882-7368-48C4-91CF-53A450C8E0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,17 +79,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>150628</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>189571</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>17066</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>132262</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Resim 2">
+        <xdr:cNvPr id="2" name="Resim 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24B9654B-92DF-32B6-2AA8-6ACC84647DE6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2942B307-67AA-A83C-F149-9D6FECBE8DE0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -106,7 +106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="14171428" cy="7428571"/>
+          <a:ext cx="15866666" cy="8704762"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Fix: Remove old DCS_A and DCS_B references from file watcher
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626D5882-7368-48C4-91CF-53A450C8E0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3335A038-299C-4EE3-BD2F-132D67B4CF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,17 +79,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>17066</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>132262</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>521905</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>84690</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Resim 1">
+        <xdr:cNvPr id="3" name="Resim 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2942B307-67AA-A83C-F149-9D6FECBE8DE0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63ABC6AA-7CC1-883F-ACBB-2661D4E3C4A6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -106,7 +106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="15866666" cy="8704762"/>
+          <a:ext cx="15761905" cy="8276190"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Excel zoom duzeltmeleri: config'den baslangic degeri, mobil duyuru arama duzeltmesi
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1959C84-EF1A-4E27-841C-3F339EC84212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172D8809-C87F-42D8-A51E-BA857DC915F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2430" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,16 +80,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>607619</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>84643</xdr:rowOff>
+      <xdr:colOff>540952</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>75167</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Resim 1">
+        <xdr:cNvPr id="3" name="Resim 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9994C3B1-F15A-EB4B-31B3-8752AA823D84}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCD2EFDB-9C5D-81C6-3259-4CDC2EE3458C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -106,7 +106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="15847619" cy="8657143"/>
+          <a:ext cx="15780952" cy="8266667"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Push notifications iyilestirmesi: mobile click support, better SW handling
</commit_message>
<xml_diff>
--- a/dcs rapor/Siparişler.xlsx
+++ b/dcs rapor/Siparişler.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berke.parlat\Desktop\ecocell\dcs rapor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172D8809-C87F-42D8-A51E-BA857DC915F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC3FD6D4-B504-476C-849C-A09FD65DA34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2430" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="2" r:id="rId1"/>
@@ -74,15 +74,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>8</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>540952</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>75167</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>333508</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>151500</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -105,8 +105,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="15780952" cy="8266667"/>
+          <a:off x="8" y="0"/>
+          <a:ext cx="13744700" cy="7200000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>